<commit_message>
Febrero con Alcon estable, falta certificacion gerentes muestra a enero
</commit_message>
<xml_diff>
--- a/datos/salida/Indicadores_Operacion.xlsx
+++ b/datos/salida/Indicadores_Operacion.xlsx
@@ -8236,63 +8236,9 @@
         <v>0.01164111300397497</v>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>LDC FC SITIO DE CONTENIDOS</t>
-        </is>
-      </c>
-      <c r="B117" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C117" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D117" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E117" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>GCIA APRENDIZAJE</t>
-        </is>
-      </c>
-      <c r="B118" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C118" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D118" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E118" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Total general</t>
-        </is>
-      </c>
-      <c r="B119" s="1" t="n">
-        <v>10372</v>
-      </c>
-      <c r="C119" s="1" t="n">
-        <v>69</v>
-      </c>
-      <c r="D119" s="1" t="n">
-        <v>10303</v>
-      </c>
-      <c r="E119" s="2" t="n">
-        <v>0.006652526031623585</v>
-      </c>
-    </row>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
     <row r="120"/>
     <row r="121"/>
     <row r="122"/>

</xml_diff>